<commit_message>
Remove DEF_TYPE column from DR escalation Excel report
</commit_message>
<xml_diff>
--- a/backend/templates/escalation_formats.xlsx
+++ b/backend/templates/escalation_formats.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="101">
   <si>
     <t>DIVISION NAME</t>
   </si>
@@ -1003,7 +1003,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1017,10 +1017,9 @@
     <col min="9" max="9" width="9.42578125" customWidth="1"/>
     <col min="10" max="10" width="17.85546875" customWidth="1"/>
     <col min="11" max="11" width="9.5703125" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -1053,9 +1052,6 @@
       </c>
       <c r="K1" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1070,7 +1066,6 @@
       <c r="I2" s="5"/>
       <c r="J2" s="6"/>
       <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>